<commit_message>
Update automation test framework
</commit_message>
<xml_diff>
--- a/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
+++ b/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -647,7 +647,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790760300682) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790763352519) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -657,30 +657,30 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Create_1790760300682</t>
+          <t>Project name: ToolsQA_Create_1790763352519</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Create_1790760300682'
-3. Verify 'ToolsQA_Create_1790760300682' appears in the project list
-4. Clean up: delete 'ToolsQA_Create_1790760300682'</t>
+2. Create a project named 'ToolsQA_Create_1790763352519'
+3. Verify 'ToolsQA_Create_1790763352519' appears in the project list
+4. Clean up: delete 'ToolsQA_Create_1790763352519'</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790760300682) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790763352519) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with name 'ToolsQA_Create_1790760300682' correctly added it to the list (cleanup delete succeeded=True).</t>
+          <t>Creating a project with name 'ToolsQA_Create_1790763352519' correctly added it to the list (cleanup delete succeeded=True).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>[PASS] New project 'ToolsQA_Create_1790760300682' appears in the list after Save</t>
+          <t>[PASS] New project 'ToolsQA_Create_1790763352519' appears in the list after Save</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790760311890), then using its 'Edit' action to change the name to ToolsQA_Rename_1790760311890_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790763364081), then using its 'Edit' action to change the name to ToolsQA_Rename_1790763364081_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -717,26 +717,26 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Original: ToolsQA_Rename_1790760311890 -&gt; Renamed: ToolsQA_Rename_1790760311890_RENAMED</t>
+          <t>Original: ToolsQA_Rename_1790763364081 -&gt; Renamed: ToolsQA_Rename_1790763364081_RENAMED</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Rename_1790760311890'
-3. Edit it, change the name to 'ToolsQA_Rename_1790760311890_RENAMED', click Update
-4. Verify 'ToolsQA_Rename_1790760311890_RENAMED' appears and 'ToolsQA_Rename_1790760311890' no longer does
-5. Clean up: delete 'ToolsQA_Rename_1790760311890_RENAMED'</t>
+2. Create a project named 'ToolsQA_Rename_1790763364081'
+3. Edit it, change the name to 'ToolsQA_Rename_1790763364081_RENAMED', click Update
+4. Verify 'ToolsQA_Rename_1790763364081_RENAMED' appears and 'ToolsQA_Rename_1790763364081' no longer does
+5. Clean up: delete 'ToolsQA_Rename_1790763364081_RENAMED'</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790760311890), then using its 'Edit' action to change the name to ToolsQA_Rename_1790760311890_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790763364081), then using its 'Edit' action to change the name to ToolsQA_Rename_1790763364081_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Renaming 'ToolsQA_Rename_1790760311890' to 'ToolsQA_Rename_1790760311890_RENAMED' correctly updated the project list.</t>
+          <t>Renaming 'ToolsQA_Rename_1790763364081' to 'ToolsQA_Rename_1790763364081_RENAMED' correctly updated the project list.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790760326907), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790763380173), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -778,26 +778,26 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_CancelDelete_1790760326907</t>
+          <t>Project name: ToolsQA_CancelDelete_1790763380173</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_CancelDelete_1790760326907'
+2. Create a project named 'ToolsQA_CancelDelete_1790763380173'
 3. Click Delete, then Cancel on the confirmation dialog
-4. Verify 'ToolsQA_CancelDelete_1790760326907' still exists
-5. Clean up: delete 'ToolsQA_CancelDelete_1790760326907' for real</t>
+4. Verify 'ToolsQA_CancelDelete_1790763380173' still exists
+5. Clean up: delete 'ToolsQA_CancelDelete_1790763380173' for real</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790760326907), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790763380173), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790760326907' correctly left it in the project list.</t>
+          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790763380173' correctly left it in the project list.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -865,6 +865,559 @@
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Projects_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project sends the real CreateProject API call and response</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790763400778) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_CreateNet_1790763400778</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project', fill 'ToolsQA_CreateNet_1790763400778'
+3. Click Save while capturing the CreateProject network call
+4. Verify method, endpoint, status 200 and response body shape
+5. Clean up: delete 'ToolsQA_CreateNet_1790763400778'</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790763400778) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Creating 'ToolsQA_CreateNet_1790763400778' fired the expected CreateProject POST and returned {'id': 3439, 'hasError': False}.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] CreateProject network call and response match the confirmed-live API shape</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Projects_08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Renaming a project sends the real RenameProject API call and response</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Editing a project (ToolsQA_RenameNet_1790763411294 -&gt; ToolsQA_RenameNet_1790763411294_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Original: ToolsQA_RenameNet_1790763411294 -&gt; Renamed: ToolsQA_RenameNet_1790763411294_UPD</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_RenameNet_1790763411294'
+3. Edit it, change the name to 'ToolsQA_RenameNet_1790763411294_UPD', click Update while capturing the network call
+4. Verify method, endpoint, status 200 and response body shape
+5. Clean up: delete 'ToolsQA_RenameNet_1790763411294_UPD'</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Editing a project (ToolsQA_RenameNet_1790763411294 -&gt; ToolsQA_RenameNet_1790763411294_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Renaming 'ToolsQA_RenameNet_1790763411294' to 'ToolsQA_RenameNet_1790763411294_UPD' fired the expected RenameProject POST and returned {'id': 3440, 'hasError': False}.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] RenameProject network call and response match the confirmed-live API shape</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Projects_09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project sends the real Delete API call and actually removes it</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790763425724) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_DeleteNet_1790763425724</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_DeleteNet_1790763425724'
+3. Delete it while capturing the Delete request and the follow-up GetProjects response
+4. Verify status 200 and the project's real absence from GetProjects</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790763425724) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting 'ToolsQA_DeleteNet_1790763425724' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Delete fired a 200 POST and the project is genuinely absent from GetProjects</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Projects_10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A whitespace-only project name is NOT treated as empty by Save's validation</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with only spaces ('   ') is confirmed live to leave Save ENABLED (only a fully empty string disables it), and the backend accepts it, creating a project with a literally blank-looking title. This is documented here as a real, live-confirmed gap - the disabled-Save validation signal is not whitespace-aware - not silently treated as a pass.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Project name: '   ' (3 spaces)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project', fill '   ' (whitespace only)
+3. Verify Save is enabled for whitespace-only input
+4. Save it and verify a project was actually created
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with only spaces ('   ') is confirmed live to leave Save ENABLED (only a fully empty string disables it), and the backend accepts it, creating a project with a literally blank-looking title. This is documented here as a real, live-confirmed gap - the disabled-Save validation signal is not whitespace-aware - not silently treated as a pass.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Whitespace-only ('   ') was correctly documented as NOT blocked: Save stayed enabled and the backend created the project - a real, live-confirmed validation gap.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Save is enabled for a whitespace-only name (not treated as empty - documented gap)
+[PASS] A whitespace-only name was accepted end-to-end (backend + list) - documented gap, not a pass we're papering over</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Projects_11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Leading/trailing whitespace on an otherwise-valid name is preserved verbatim</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790763447994  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Project name (with padding): '  ToolsQA_Whitespace_1790763447994  '</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named '  ToolsQA_Whitespace_1790763447994  '
+3. Verify the CreateProject payload/response preserved the padding verbatim
+4. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790763447994  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>The padded name '  ToolsQA_Whitespace_1790763447994  ' was saved and listed exactly as typed, with no trimming applied.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Leading/trailing whitespace in the name was preserved verbatim (not trimmed)</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Projects_12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>A very long (300-char class) project name has no enforced client/server limit</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed live: the 'Project Name' input has no HTML 'maxlength' attribute, and a 300-character name is accepted verbatim by both the input and the backend (CreateProject responds hasError=false, no truncation/rejection). Documented as a real, live-confirmed gap - no length limit is enforced anywhere in this flow.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Project name length: 287 chars</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project'
+3. Verify the name input has no 'maxlength' attribute
+4. Fill a 287-char name and Save; verify it's accepted untruncated
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed live: the 'Project Name' input has no HTML 'maxlength' attribute, and a 300-character name is accepted verbatim by both the input and the backend (CreateProject responds hasError=false, no truncation/rejection). Documented as a real, live-confirmed gap - no length limit is enforced anywhere in this flow.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>A 287-char name was correctly accepted with no length limit enforced anywhere in the flow.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The 'Project Name' input has no 'maxlength' attribute (documented gap)
+[PASS] A 300-char-class name was accepted untruncated, client and server side</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Projects_13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A true duplicate project name is blocked server-side, but with no visible user feedback</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790763470408') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Project name (used twice): ToolsQA_Dup_1790763470408</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Dup_1790763470408'
+3. Attempt to create a second project with the exact same name
+4. Verify the backend rejected the duplicate (hasError=true) and no visible error feedback is shown to the user
+5. Verify only one row with this title exists
+6. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790763470408') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate creation of 'ToolsQA_Dup_1790763470408' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] CreateProject correctly rejected the exact-duplicate name (data-level protection)
+[PASS] No toast/inline error is shown to the user for the rejected duplicate (documented UX gap)
+[PASS] No duplicate row was actually created despite the silent UI failure</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Projects_14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>A special-character/XSS-style project name saves and renders safely</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Project name: &lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;'
+3. Verify it was saved and is displayed as visible text
+4. Verify no live '&lt;script&gt;' tag was injected into the page HTML
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>'&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The special-character name is saved and rendered as visible text
+[PASS] No live '&lt;script&gt;' tag was injected (safe/escaped rendering, not a real XSS)</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Projects_15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>A newly created project survives a page reload (real server persistence)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>After creating a project ('ToolsQA_Persist_1790763496928'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_Persist_1790763496928</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Persist_1790763496928'
+3. Reload the page
+4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790763496928' is still listed
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>After creating a project ('ToolsQA_Persist_1790763496928'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>'ToolsQA_Persist_1790763496928' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The created project survived a reload (real server persistence, no redirect-away)</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
chore: refresh test_data Excel files from full-suite verification run (166/166 passed)
</commit_message>
<xml_diff>
--- a/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
+++ b/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790763352519) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790766514936) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -657,30 +657,30 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Create_1790763352519</t>
+          <t>Project name: ToolsQA_Create_1790766514936</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Create_1790763352519'
-3. Verify 'ToolsQA_Create_1790763352519' appears in the project list
-4. Clean up: delete 'ToolsQA_Create_1790763352519'</t>
+2. Create a project named 'ToolsQA_Create_1790766514936'
+3. Verify 'ToolsQA_Create_1790766514936' appears in the project list
+4. Clean up: delete 'ToolsQA_Create_1790766514936'</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790763352519) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790766514936) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with name 'ToolsQA_Create_1790763352519' correctly added it to the list (cleanup delete succeeded=True).</t>
+          <t>Creating a project with name 'ToolsQA_Create_1790766514936' correctly added it to the list (cleanup delete succeeded=True).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>[PASS] New project 'ToolsQA_Create_1790763352519' appears in the list after Save</t>
+          <t>[PASS] New project 'ToolsQA_Create_1790766514936' appears in the list after Save</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790763364081), then using its 'Edit' action to change the name to ToolsQA_Rename_1790763364081_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790766527149), then using its 'Edit' action to change the name to ToolsQA_Rename_1790766527149_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -717,26 +717,26 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Original: ToolsQA_Rename_1790763364081 -&gt; Renamed: ToolsQA_Rename_1790763364081_RENAMED</t>
+          <t>Original: ToolsQA_Rename_1790766527149 -&gt; Renamed: ToolsQA_Rename_1790766527149_RENAMED</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Rename_1790763364081'
-3. Edit it, change the name to 'ToolsQA_Rename_1790763364081_RENAMED', click Update
-4. Verify 'ToolsQA_Rename_1790763364081_RENAMED' appears and 'ToolsQA_Rename_1790763364081' no longer does
-5. Clean up: delete 'ToolsQA_Rename_1790763364081_RENAMED'</t>
+2. Create a project named 'ToolsQA_Rename_1790766527149'
+3. Edit it, change the name to 'ToolsQA_Rename_1790766527149_RENAMED', click Update
+4. Verify 'ToolsQA_Rename_1790766527149_RENAMED' appears and 'ToolsQA_Rename_1790766527149' no longer does
+5. Clean up: delete 'ToolsQA_Rename_1790766527149_RENAMED'</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790763364081), then using its 'Edit' action to change the name to ToolsQA_Rename_1790763364081_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790766527149), then using its 'Edit' action to change the name to ToolsQA_Rename_1790766527149_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Renaming 'ToolsQA_Rename_1790763364081' to 'ToolsQA_Rename_1790763364081_RENAMED' correctly updated the project list.</t>
+          <t>Renaming 'ToolsQA_Rename_1790766527149' to 'ToolsQA_Rename_1790766527149_RENAMED' correctly updated the project list.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790763380173), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790766542615), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -778,26 +778,26 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_CancelDelete_1790763380173</t>
+          <t>Project name: ToolsQA_CancelDelete_1790766542615</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_CancelDelete_1790763380173'
+2. Create a project named 'ToolsQA_CancelDelete_1790766542615'
 3. Click Delete, then Cancel on the confirmation dialog
-4. Verify 'ToolsQA_CancelDelete_1790763380173' still exists
-5. Clean up: delete 'ToolsQA_CancelDelete_1790763380173' for real</t>
+4. Verify 'ToolsQA_CancelDelete_1790766542615' still exists
+5. Clean up: delete 'ToolsQA_CancelDelete_1790766542615' for real</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790763380173), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790766542615), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790763380173' correctly left it in the project list.</t>
+          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790766542615' correctly left it in the project list.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790763400778) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790766565055) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -898,26 +898,26 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_CreateNet_1790763400778</t>
+          <t>Project name: ToolsQA_CreateNet_1790766565055</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Open 'New Project', fill 'ToolsQA_CreateNet_1790763400778'
+2. Open 'New Project', fill 'ToolsQA_CreateNet_1790766565055'
 3. Click Save while capturing the CreateProject network call
 4. Verify method, endpoint, status 200 and response body shape
-5. Clean up: delete 'ToolsQA_CreateNet_1790763400778'</t>
+5. Clean up: delete 'ToolsQA_CreateNet_1790766565055'</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790763400778) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790766565055) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Creating 'ToolsQA_CreateNet_1790763400778' fired the expected CreateProject POST and returned {'id': 3439, 'hasError': False}.</t>
+          <t>Creating 'ToolsQA_CreateNet_1790766565055' fired the expected CreateProject POST and returned {'id': 3478, 'hasError': False}.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Editing a project (ToolsQA_RenameNet_1790763411294 -&gt; ToolsQA_RenameNet_1790763411294_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+          <t>Editing a project (ToolsQA_RenameNet_1790766576994 -&gt; ToolsQA_RenameNet_1790766576994_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -959,26 +959,26 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Original: ToolsQA_RenameNet_1790763411294 -&gt; Renamed: ToolsQA_RenameNet_1790763411294_UPD</t>
+          <t>Original: ToolsQA_RenameNet_1790766576994 -&gt; Renamed: ToolsQA_RenameNet_1790766576994_UPD</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_RenameNet_1790763411294'
-3. Edit it, change the name to 'ToolsQA_RenameNet_1790763411294_UPD', click Update while capturing the network call
+2. Create a project named 'ToolsQA_RenameNet_1790766576994'
+3. Edit it, change the name to 'ToolsQA_RenameNet_1790766576994_UPD', click Update while capturing the network call
 4. Verify method, endpoint, status 200 and response body shape
-5. Clean up: delete 'ToolsQA_RenameNet_1790763411294_UPD'</t>
+5. Clean up: delete 'ToolsQA_RenameNet_1790766576994_UPD'</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Editing a project (ToolsQA_RenameNet_1790763411294 -&gt; ToolsQA_RenameNet_1790763411294_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+          <t>Editing a project (ToolsQA_RenameNet_1790766576994 -&gt; ToolsQA_RenameNet_1790766576994_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Renaming 'ToolsQA_RenameNet_1790763411294' to 'ToolsQA_RenameNet_1790763411294_UPD' fired the expected RenameProject POST and returned {'id': 3440, 'hasError': False}.</t>
+          <t>Renaming 'ToolsQA_RenameNet_1790766576994' to 'ToolsQA_RenameNet_1790766576994_UPD' fired the expected RenameProject POST and returned {'id': 3479, 'hasError': False}.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Deleting a project (ToolsQA_DeleteNet_1790763425724) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790766592899) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1020,25 +1020,25 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_DeleteNet_1790763425724</t>
+          <t>Project name: ToolsQA_DeleteNet_1790766592899</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_DeleteNet_1790763425724'
+2. Create a project named 'ToolsQA_DeleteNet_1790766592899'
 3. Delete it while capturing the Delete request and the follow-up GetProjects response
 4. Verify status 200 and the project's real absence from GetProjects</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Deleting a project (ToolsQA_DeleteNet_1790763425724) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790766592899) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Deleting 'ToolsQA_DeleteNet_1790763425724' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
+          <t>Deleting 'ToolsQA_DeleteNet_1790766592899' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790763447994  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790766617768  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1142,25 +1142,25 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Project name (with padding): '  ToolsQA_Whitespace_1790763447994  '</t>
+          <t>Project name (with padding): '  ToolsQA_Whitespace_1790766617768  '</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named '  ToolsQA_Whitespace_1790763447994  '
+2. Create a project named '  ToolsQA_Whitespace_1790766617768  '
 3. Verify the CreateProject payload/response preserved the padding verbatim
 4. Clean up: delete it</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790763447994  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790766617768  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>The padded name '  ToolsQA_Whitespace_1790763447994  ' was saved and listed exactly as typed, with no trimming applied.</t>
+          <t>The padded name '  ToolsQA_Whitespace_1790766617768  ' was saved and listed exactly as typed, with no trimming applied.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790763470408') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790766643303') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1264,13 +1264,13 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Project name (used twice): ToolsQA_Dup_1790763470408</t>
+          <t>Project name (used twice): ToolsQA_Dup_1790766643303</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Dup_1790763470408'
+2. Create a project named 'ToolsQA_Dup_1790766643303'
 3. Attempt to create a second project with the exact same name
 4. Verify the backend rejected the duplicate (hasError=true) and no visible error feedback is shown to the user
 5. Verify only one row with this title exists
@@ -1279,12 +1279,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790763470408') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790766643303') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Duplicate creation of 'ToolsQA_Dup_1790763470408' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
+          <t>Duplicate creation of 'ToolsQA_Dup_1790766643303' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790766658916')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,13 +1328,13 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Project name: &lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;</t>
+          <t>Project name: &lt;script&gt;alert('ToolsQA_1790766658916')&lt;/script&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;'
+2. Create a project named '&lt;script&gt;alert('ToolsQA_1790766658916')&lt;/script&gt;'
 3. Verify it was saved and is displayed as visible text
 4. Verify no live '&lt;script&gt;' tag was injected into the page HTML
 5. Clean up: delete it</t>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790766658916')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>'&lt;script&gt;alert('ToolsQA_1790763484700')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
+          <t>'&lt;script&gt;alert('ToolsQA_1790766658916')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>After creating a project ('ToolsQA_Persist_1790763496928'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+          <t>After creating a project ('ToolsQA_Persist_1790766672903'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1390,26 +1390,26 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Persist_1790763496928</t>
+          <t>Project name: ToolsQA_Persist_1790766672903</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Persist_1790763496928'
+2. Create a project named 'ToolsQA_Persist_1790766672903'
 3. Reload the page
-4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790763496928' is still listed
+4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790766672903' is still listed
 5. Clean up: delete it</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>After creating a project ('ToolsQA_Persist_1790763496928'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+          <t>After creating a project ('ToolsQA_Persist_1790766672903'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>'ToolsQA_Persist_1790763496928' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
+          <t>'ToolsQA_Persist_1790766672903' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: refresh test_data Excel files from final 189/189 verification run
</commit_message>
<xml_diff>
--- a/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
+++ b/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -512,59 +512,973 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Projects_01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Projects page loads with the project list and 'New Project' control</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>The page must load at /wta/Project with the 'New Project' button visible and at least one existing project listed (this account has prior saved projects).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Verify URL and 'New Project' button
+3. Verify at least one existing project row is visible</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>The page must load at /wta/Project with the 'New Project' button visible and at least one existing project listed (this account has prior saved projects).</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Projects loaded correctly at https://regplus.kaz.com.bd/wta/Project with existing projects listed.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Projects page loads with 'New Project' and an existing project list</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Projects_02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>'New Project' Save is disabled until a project name is entered</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Opening 'New Project' with a blank 'Project Name' field must leave the Save button disabled (the app's client-side validation for a required field), and Cancel must close the modal without creating any project.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project'
+3. Verify Save is disabled with an empty name
+4. Click Cancel and verify the modal closes</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Opening 'New Project' with a blank 'Project Name' field must leave the Save button disabled (the app's client-side validation for a required field), and Cancel must close the modal without creating any project.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>'New Project' correctly disabled Save for a blank name and Cancel closed the modal.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Save button is disabled while the project name is empty
+[PASS] Save was disabled for a blank name and Cancel closed the modal</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Projects_03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Creating a new project adds it to the project list</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790770510429) and clicking Save must add a new project with that exact title to the list.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_Create_1790770510429</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Create_1790770510429'
+3. Verify 'ToolsQA_Create_1790770510429' appears in the project list
+4. Clean up: delete 'ToolsQA_Create_1790770510429'</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790770510429) and clicking Save must add a new project with that exact title to the list.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project with name 'ToolsQA_Create_1790770510429' correctly added it to the list (cleanup delete succeeded=True).</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] New project 'ToolsQA_Create_1790770510429' appears in the list after Save</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Projects_04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Editing a project renames it (Update)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project (ToolsQA_Rename_1790770523146), then using its 'Edit' action to change the name to ToolsQA_Rename_1790770523146_RENAMED and clicking Update must replace the title in the list.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Original: ToolsQA_Rename_1790770523146 -&gt; Renamed: ToolsQA_Rename_1790770523146_RENAMED</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Rename_1790770523146'
+3. Edit it, change the name to 'ToolsQA_Rename_1790770523146_RENAMED', click Update
+4. Verify 'ToolsQA_Rename_1790770523146_RENAMED' appears and 'ToolsQA_Rename_1790770523146' no longer does
+5. Clean up: delete 'ToolsQA_Rename_1790770523146_RENAMED'</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project (ToolsQA_Rename_1790770523146), then using its 'Edit' action to change the name to ToolsQA_Rename_1790770523146_RENAMED and clicking Update must replace the title in the list.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Renaming 'ToolsQA_Rename_1790770523146' to 'ToolsQA_Rename_1790770523146_RENAMED' correctly updated the project list.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Renaming a project updates its title in the list</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Projects_05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Cancelling the delete confirmation keeps the project</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project (ToolsQA_CancelDelete_1790770539359), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_CancelDelete_1790770539359</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_CancelDelete_1790770539359'
+3. Click Delete, then Cancel on the confirmation dialog
+4. Verify 'ToolsQA_CancelDelete_1790770539359' still exists
+5. Clean up: delete 'ToolsQA_CancelDelete_1790770539359' for real</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project (ToolsQA_CancelDelete_1790770539359), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790770539359' correctly left it in the project list.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Cancelling the delete confirmation left the project in place</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Projects_06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Selecting an existing project shows its item table</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Clicking an existing project's title must switch the detail pane to a table with the confirmed columns: '#', 'Title', 'Description', 'Jurisdiction', 'Type'.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects, with at least one existing project.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Click the first existing project's title
+3. Verify the detail table shows the expected columns</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Clicking an existing project's title must switch the detail pane to a table with the confirmed columns: '#', 'Title', 'Description', 'Jurisdiction', 'Type'.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Selecting a project correctly showed its item table with headers ['', '#', 'Title', 'Description', 'Jurisdiction', 'Type', ''].</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Project detail table shows the expected columns</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Projects_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project sends the real CreateProject API call and response</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790770562641) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_CreateNet_1790770562641</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project', fill 'ToolsQA_CreateNet_1790770562641'
+3. Click Save while capturing the CreateProject network call
+4. Verify method, endpoint, status 200 and response body shape
+5. Clean up: delete 'ToolsQA_CreateNet_1790770562641'</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790770562641) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Creating 'ToolsQA_CreateNet_1790770562641' fired the expected CreateProject POST and returned {'id': 3493, 'hasError': False}.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] CreateProject network call and response match the confirmed-live API shape</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Projects_08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Renaming a project sends the real RenameProject API call and response</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Editing a project (ToolsQA_RenameNet_1790770573089 -&gt; ToolsQA_RenameNet_1790770573089_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Original: ToolsQA_RenameNet_1790770573089 -&gt; Renamed: ToolsQA_RenameNet_1790770573089_UPD</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_RenameNet_1790770573089'
+3. Edit it, change the name to 'ToolsQA_RenameNet_1790770573089_UPD', click Update while capturing the network call
+4. Verify method, endpoint, status 200 and response body shape
+5. Clean up: delete 'ToolsQA_RenameNet_1790770573089_UPD'</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Editing a project (ToolsQA_RenameNet_1790770573089 -&gt; ToolsQA_RenameNet_1790770573089_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Renaming 'ToolsQA_RenameNet_1790770573089' to 'ToolsQA_RenameNet_1790770573089_UPD' fired the expected RenameProject POST and returned {'id': 3494, 'hasError': False}.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] RenameProject network call and response match the confirmed-live API shape</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Projects_09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project sends the real Delete API call and actually removes it</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790770587859) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_DeleteNet_1790770587859</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_DeleteNet_1790770587859'
+3. Delete it while capturing the Delete request and the follow-up GetProjects response
+4. Verify status 200 and the project's real absence from GetProjects</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790770587859) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Deleting 'ToolsQA_DeleteNet_1790770587859' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Delete fired a 200 POST and the project is genuinely absent from GetProjects</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Projects_10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A whitespace-only project name is NOT treated as empty by Save's validation</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with only spaces ('   ') is confirmed live to leave Save ENABLED (only a fully empty string disables it), and the backend accepts it, creating a project with a literally blank-looking title. This is documented here as a real, live-confirmed gap - the disabled-Save validation signal is not whitespace-aware - not silently treated as a pass.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Project name: '   ' (3 spaces)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project', fill '   ' (whitespace only)
+3. Verify Save is enabled for whitespace-only input
+4. Save it and verify a project was actually created
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Filling 'Project Name' with only spaces ('   ') is confirmed live to leave Save ENABLED (only a fully empty string disables it), and the backend accepts it, creating a project with a literally blank-looking title. This is documented here as a real, live-confirmed gap - the disabled-Save validation signal is not whitespace-aware - not silently treated as a pass.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Whitespace-only ('   ') was correctly documented as NOT blocked: Save stayed enabled and the backend created the project - a real, live-confirmed validation gap.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Save is enabled for a whitespace-only name (not treated as empty - documented gap)
+[PASS] A whitespace-only name was accepted end-to-end (backend + list) - documented gap, not a pass we're papering over</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Projects_11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Leading/trailing whitespace on an otherwise-valid name is preserved verbatim</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790770611080  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Project name (with padding): '  ToolsQA_Whitespace_1790770611080  '</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named '  ToolsQA_Whitespace_1790770611080  '
+3. Verify the CreateProject payload/response preserved the padding verbatim
+4. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790770611080  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>The padded name '  ToolsQA_Whitespace_1790770611080  ' was saved and listed exactly as typed, with no trimming applied.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Leading/trailing whitespace in the name was preserved verbatim (not trimmed)</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Projects_12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>A very long (300-char class) project name has no enforced client/server limit</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed live: the 'Project Name' input has no HTML 'maxlength' attribute, and a 300-character name is accepted verbatim by both the input and the backend (CreateProject responds hasError=false, no truncation/rejection). Documented as a real, live-confirmed gap - no length limit is enforced anywhere in this flow.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Project name length: 287 chars</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Open 'New Project'
+3. Verify the name input has no 'maxlength' attribute
+4. Fill a 287-char name and Save; verify it's accepted untruncated
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed live: the 'Project Name' input has no HTML 'maxlength' attribute, and a 300-character name is accepted verbatim by both the input and the backend (CreateProject responds hasError=false, no truncation/rejection). Documented as a real, live-confirmed gap - no length limit is enforced anywhere in this flow.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>A 287-char name was correctly accepted with no length limit enforced anywhere in the flow.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The 'Project Name' input has no 'maxlength' attribute (documented gap)
+[PASS] A 300-char-class name was accepted untruncated, client and server side</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Projects_13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A true duplicate project name is blocked server-side, but with no visible user feedback</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790770634549') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Project name (used twice): ToolsQA_Dup_1790770634549</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Dup_1790770634549'
+3. Attempt to create a second project with the exact same name
+4. Verify the backend rejected the duplicate (hasError=true) and no visible error feedback is shown to the user
+5. Verify only one row with this title exists
+6. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790770634549') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate creation of 'ToolsQA_Dup_1790770634549' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] CreateProject correctly rejected the exact-duplicate name (data-level protection)
+[PASS] No toast/inline error is shown to the user for the rejected duplicate (documented UX gap)
+[PASS] No duplicate row was actually created despite the silent UI failure</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Projects_14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>A special-character/XSS-style project name saves and renders safely</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Project name: &lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;'
+3. Verify it was saved and is displayed as visible text
+4. Verify no live '&lt;script&gt;' tag was injected into the page HTML
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>'&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The special-character name is saved and rendered as visible text
+[PASS] No live '&lt;script&gt;' tag was injected (safe/escaped rendering, not a real XSS)</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Projects_15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>A newly created project survives a page reload (real server persistence)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>After creating a project ('ToolsQA_Persist_1790770661553'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Tools &gt; Projects.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_Persist_1790770661553</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Persist_1790770661553'
+3. Reload the page
+4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790770661553' is still listed
+5. Clean up: delete it</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>After creating a project ('ToolsQA_Persist_1790770661553'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>'ToolsQA_Persist_1790770661553' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The created project survived a reload (real server persistence, no redirect-away)</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Projects_16</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Tools Projects</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Tools Projects</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>A project row's 'Export' action downloads a real, non-empty file</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770149620').</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770675458').</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Tools &gt; Projects.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Project name: ToolsQA_Export_1790770149620</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Export_1790770149620'
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Project name: ToolsQA_Export_1790770675458</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Tools &gt; Projects
+2. Create a project named 'ToolsQA_Export_1790770675458'
 3. Hover the row and click its 'Export' action
 4. Verify a real, non-empty file download completed
 5. Clean up: delete it</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770149620').</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>The 'Export' action correctly downloaded 'ToolsQA_Export_1790770149620.xlsx' (2951 bytes).</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770675458').</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>The 'Export' action correctly downloaded 'ToolsQA_Export_1790770675458.xlsx' (2952 bytes).</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>[PASS] The row's 'Export' action produces a real, non-empty file with no failure</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
chore: refresh test_data Excel files from full-suite verification run (190/190 passed)
</commit_message>
<xml_diff>
--- a/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
+++ b/test_data/Tools Projects/Tools Projects_Test_Cases.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790770510429) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790771839655) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -657,30 +657,30 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Create_1790770510429</t>
+          <t>Project name: ToolsQA_Create_1790771839655</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Create_1790770510429'
-3. Verify 'ToolsQA_Create_1790770510429' appears in the project list
-4. Clean up: delete 'ToolsQA_Create_1790770510429'</t>
+2. Create a project named 'ToolsQA_Create_1790771839655'
+3. Verify 'ToolsQA_Create_1790771839655' appears in the project list
+4. Clean up: delete 'ToolsQA_Create_1790771839655'</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790770510429) and clicking Save must add a new project with that exact title to the list.</t>
+          <t>Filling 'Project Name' with a unique title (ToolsQA_Create_1790771839655) and clicking Save must add a new project with that exact title to the list.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with name 'ToolsQA_Create_1790770510429' correctly added it to the list (cleanup delete succeeded=True).</t>
+          <t>Creating a project with name 'ToolsQA_Create_1790771839655' correctly added it to the list (cleanup delete succeeded=True).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>[PASS] New project 'ToolsQA_Create_1790770510429' appears in the list after Save</t>
+          <t>[PASS] New project 'ToolsQA_Create_1790771839655' appears in the list after Save</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790770523146), then using its 'Edit' action to change the name to ToolsQA_Rename_1790770523146_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790771851332), then using its 'Edit' action to change the name to ToolsQA_Rename_1790771851332_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -717,26 +717,26 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Original: ToolsQA_Rename_1790770523146 -&gt; Renamed: ToolsQA_Rename_1790770523146_RENAMED</t>
+          <t>Original: ToolsQA_Rename_1790771851332 -&gt; Renamed: ToolsQA_Rename_1790771851332_RENAMED</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Rename_1790770523146'
-3. Edit it, change the name to 'ToolsQA_Rename_1790770523146_RENAMED', click Update
-4. Verify 'ToolsQA_Rename_1790770523146_RENAMED' appears and 'ToolsQA_Rename_1790770523146' no longer does
-5. Clean up: delete 'ToolsQA_Rename_1790770523146_RENAMED'</t>
+2. Create a project named 'ToolsQA_Rename_1790771851332'
+3. Edit it, change the name to 'ToolsQA_Rename_1790771851332_RENAMED', click Update
+4. Verify 'ToolsQA_Rename_1790771851332_RENAMED' appears and 'ToolsQA_Rename_1790771851332' no longer does
+5. Clean up: delete 'ToolsQA_Rename_1790771851332_RENAMED'</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_Rename_1790770523146), then using its 'Edit' action to change the name to ToolsQA_Rename_1790770523146_RENAMED and clicking Update must replace the title in the list.</t>
+          <t>Creating a project (ToolsQA_Rename_1790771851332), then using its 'Edit' action to change the name to ToolsQA_Rename_1790771851332_RENAMED and clicking Update must replace the title in the list.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Renaming 'ToolsQA_Rename_1790770523146' to 'ToolsQA_Rename_1790770523146_RENAMED' correctly updated the project list.</t>
+          <t>Renaming 'ToolsQA_Rename_1790771851332' to 'ToolsQA_Rename_1790771851332_RENAMED' correctly updated the project list.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790770539359), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790771866844), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -778,26 +778,26 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_CancelDelete_1790770539359</t>
+          <t>Project name: ToolsQA_CancelDelete_1790771866844</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_CancelDelete_1790770539359'
+2. Create a project named 'ToolsQA_CancelDelete_1790771866844'
 3. Click Delete, then Cancel on the confirmation dialog
-4. Verify 'ToolsQA_CancelDelete_1790770539359' still exists
-5. Clean up: delete 'ToolsQA_CancelDelete_1790770539359' for real</t>
+4. Verify 'ToolsQA_CancelDelete_1790771866844' still exists
+5. Clean up: delete 'ToolsQA_CancelDelete_1790771866844' for real</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Creating a project (ToolsQA_CancelDelete_1790770539359), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
+          <t>Creating a project (ToolsQA_CancelDelete_1790771866844), clicking its 'Delete' action, then clicking 'Cancel' on the 'Confirm Delete' dialog must leave the project in the list untouched.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790770539359' correctly left it in the project list.</t>
+          <t>Cancelling the delete confirmation for 'ToolsQA_CancelDelete_1790771866844' correctly left it in the project list.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790770562641) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790771888812) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -898,26 +898,26 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_CreateNet_1790770562641</t>
+          <t>Project name: ToolsQA_CreateNet_1790771888812</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Open 'New Project', fill 'ToolsQA_CreateNet_1790770562641'
+2. Open 'New Project', fill 'ToolsQA_CreateNet_1790771888812'
 3. Click Save while capturing the CreateProject network call
 4. Verify method, endpoint, status 200 and response body shape
-5. Clean up: delete 'ToolsQA_CreateNet_1790770562641'</t>
+5. Clean up: delete 'ToolsQA_CreateNet_1790771888812'</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790770562641) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
+          <t>Clicking Save for a new project (ToolsQA_CreateNet_1790771888812) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/CreateProject' request with the typed name, and the response must be HTTP 200 with a JSON body of the confirmed-live shape '{"id":&lt;newId&gt;,"hasError":false}' - a real, non-zero id and hasError=false.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Creating 'ToolsQA_CreateNet_1790770562641' fired the expected CreateProject POST and returned {'id': 3493, 'hasError': False}.</t>
+          <t>Creating 'ToolsQA_CreateNet_1790771888812' fired the expected CreateProject POST and returned {'id': 3507, 'hasError': False}.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Editing a project (ToolsQA_RenameNet_1790770573089 -&gt; ToolsQA_RenameNet_1790770573089_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+          <t>Editing a project (ToolsQA_RenameNet_1790771900563 -&gt; ToolsQA_RenameNet_1790771900563_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -959,26 +959,26 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Original: ToolsQA_RenameNet_1790770573089 -&gt; Renamed: ToolsQA_RenameNet_1790770573089_UPD</t>
+          <t>Original: ToolsQA_RenameNet_1790771900563 -&gt; Renamed: ToolsQA_RenameNet_1790771900563_UPD</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_RenameNet_1790770573089'
-3. Edit it, change the name to 'ToolsQA_RenameNet_1790770573089_UPD', click Update while capturing the network call
+2. Create a project named 'ToolsQA_RenameNet_1790771900563'
+3. Edit it, change the name to 'ToolsQA_RenameNet_1790771900563_UPD', click Update while capturing the network call
 4. Verify method, endpoint, status 200 and response body shape
-5. Clean up: delete 'ToolsQA_RenameNet_1790770573089_UPD'</t>
+5. Clean up: delete 'ToolsQA_RenameNet_1790771900563_UPD'</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Editing a project (ToolsQA_RenameNet_1790770573089 -&gt; ToolsQA_RenameNet_1790770573089_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
+          <t>Editing a project (ToolsQA_RenameNet_1790771900563 -&gt; ToolsQA_RenameNet_1790771900563_UPD) and clicking Update must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/RenameProject' request with the new name, and the response must be HTTP 200 with the confirmed-live shape '{"id":&lt;sameId&gt;,"hasError":false}'.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Renaming 'ToolsQA_RenameNet_1790770573089' to 'ToolsQA_RenameNet_1790770573089_UPD' fired the expected RenameProject POST and returned {'id': 3494, 'hasError': False}.</t>
+          <t>Renaming 'ToolsQA_RenameNet_1790771900563' to 'ToolsQA_RenameNet_1790771900563_UPD' fired the expected RenameProject POST and returned {'id': 3508, 'hasError': False}.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Deleting a project (ToolsQA_DeleteNet_1790770587859) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790771915278) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1020,25 +1020,25 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_DeleteNet_1790770587859</t>
+          <t>Project name: ToolsQA_DeleteNet_1790771915278</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_DeleteNet_1790770587859'
+2. Create a project named 'ToolsQA_DeleteNet_1790771915278'
 3. Delete it while capturing the Delete request and the follow-up GetProjects response
 4. Verify status 200 and the project's real absence from GetProjects</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Deleting a project (ToolsQA_DeleteNet_1790770587859) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
+          <t>Deleting a project (ToolsQA_DeleteNet_1790771915278) must fire a 'POST https://regpluswta.api.kaz.com.bd/api/Project/Delete' request with HTTP 200, and the project must be genuinely gone from the account afterwards (re-fetched via the app's own follow-up GetProjects call, not just the UI's optimistic removal). NOTE (confirmed live - see pages/tools_projects_page.py): the Delete response body shape differs from Create/Rename ('{"isSuccess":&lt;bool&gt;,"error":...}'), and 'isSuccess' has been observed to intermittently report false (an EF Core DbContext-threading error) even when the project was in fact removed - so this test treats HTTP 200 plus the project's real absence from the next GetProjects response as the authoritative pass condition, not the possibly-flaky 'isSuccess' field alone.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Deleting 'ToolsQA_DeleteNet_1790770587859' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
+          <t>Deleting 'ToolsQA_DeleteNet_1790771915278' correctly returned HTTP 200 and the project was genuinely gone from GetProjects afterwards (isSuccess reported as False).</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790770611080  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790771937246  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1142,25 +1142,25 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Project name (with padding): '  ToolsQA_Whitespace_1790770611080  '</t>
+          <t>Project name (with padding): '  ToolsQA_Whitespace_1790771937246  '</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named '  ToolsQA_Whitespace_1790770611080  '
+2. Create a project named '  ToolsQA_Whitespace_1790771937246  '
 3. Verify the CreateProject payload/response preserved the padding verbatim
 4. Clean up: delete it</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790770611080  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
+          <t>Creating a project with a name padded with leading/trailing spaces ('  ToolsQA_Whitespace_1790771937246  ') is confirmed live to be saved EXACTLY as typed - the app does not trim it client-side before enabling Save, nor server-side in storage. Documented as an observation about real app behavior, not asserted as right or wrong.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>The padded name '  ToolsQA_Whitespace_1790770611080  ' was saved and listed exactly as typed, with no trimming applied.</t>
+          <t>The padded name '  ToolsQA_Whitespace_1790771937246  ' was saved and listed exactly as typed, with no trimming applied.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790770634549') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790771961829') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1264,13 +1264,13 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Project name (used twice): ToolsQA_Dup_1790770634549</t>
+          <t>Project name (used twice): ToolsQA_Dup_1790771961829</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Dup_1790770634549'
+2. Create a project named 'ToolsQA_Dup_1790771961829'
 3. Attempt to create a second project with the exact same name
 4. Verify the backend rejected the duplicate (hasError=true) and no visible error feedback is shown to the user
 5. Verify only one row with this title exists
@@ -1279,12 +1279,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790770634549') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
+          <t>Creating a second project with the exact same name as an existing one ('ToolsQA_Dup_1790771961829') is confirmed live to be blocked at the data level - CreateProject responds '{"id":0,"hasError":true,"errorMessage":"Please choose another name"}' and no duplicate row is created. However, this is ALSO confirmed live to be a real UX gap: the modal simply closes with zero visible feedback to the user (no toast, no inline error) - the rejection is silent. Both are documented and asserted: the app correctly prevents duplicate DATA, but gives the user no correct signal that their second attempt failed.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Duplicate creation of 'ToolsQA_Dup_1790770634549' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
+          <t>Duplicate creation of 'ToolsQA_Dup_1790771961829' was correctly blocked at the data level (hasError=true, no duplicate row), but the UI gave the user no visible feedback that the attempt failed - a real, documented UX gap.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790771977345')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,13 +1328,13 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Project name: &lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;</t>
+          <t>Project name: &lt;script&gt;alert('ToolsQA_1790771977345')&lt;/script&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;'
+2. Create a project named '&lt;script&gt;alert('ToolsQA_1790771977345')&lt;/script&gt;'
 3. Verify it was saved and is displayed as visible text
 4. Verify no live '&lt;script&gt;' tag was injected into the page HTML
 5. Clean up: delete it</t>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
+          <t>Creating a project named literally '&lt;script&gt;alert('ToolsQA_1790771977345')&lt;/script&gt;' is confirmed live to save and list successfully (the backend does not reject special characters), and to render back as plain escaped text - NOT as a live '&lt;script&gt;' element in the page (0 matches for the raw tag in page HTML). This is a documented XSS-safety PASS for this field, verified live rather than assumed.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>'&lt;script&gt;alert('ToolsQA_1790770649198')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
+          <t>'&lt;script&gt;alert('ToolsQA_1790771977345')&lt;/script&gt;' saved successfully and rendered as safe, escaped text with no live script injection.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>After creating a project ('ToolsQA_Persist_1790770661553'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+          <t>After creating a project ('ToolsQA_Persist_1790771989230'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1390,26 +1390,26 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Persist_1790770661553</t>
+          <t>Project name: ToolsQA_Persist_1790771989230</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Persist_1790770661553'
+2. Create a project named 'ToolsQA_Persist_1790771989230'
 3. Reload the page
-4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790770661553' is still listed
+4. Verify the URL is still /wta/Project and 'ToolsQA_Persist_1790771989230' is still listed
 5. Clean up: delete it</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>After creating a project ('ToolsQA_Persist_1790770661553'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
+          <t>After creating a project ('ToolsQA_Persist_1790771989230'), reloading the page must still show it - proving the save is real server-side persistence, not just an optimistic client-side UI update. Confirmed live: unlike a fresh external 'page.goto("/wta/Project")' (which redirects to /wta/Information per the documented Tools deep-link gotcha), 'page.reload()' from an already-open /wta/Project page stays on /wta/Project and re-fetches the list from the server, so this test uses reload() rather than re-navigating through the Tools menu.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>'ToolsQA_Persist_1790770661553' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
+          <t>'ToolsQA_Persist_1790771989230' correctly survived a page reload, staying on https://regplus.kaz.com.bd/wta/Project - proving real server-side persistence.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770675458').</t>
+          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790772024380').</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1451,13 +1451,13 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Project name: ToolsQA_Export_1790770675458</t>
+          <t>Project name: ToolsQA_Export_1790772024380</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Tools &gt; Projects
-2. Create a project named 'ToolsQA_Export_1790770675458'
+2. Create a project named 'ToolsQA_Export_1790772024380'
 3. Hover the row and click its 'Export' action
 4. Verify a real, non-empty file download completed
 5. Clean up: delete it</t>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790770675458').</t>
+          <t>Each project row's hover-revealed 'Export' link (defined in the page object's 'row_action' helper alongside 'Edit'/'Delete', but never previously clicked by any test) must trigger a real file download with no failure and a non-zero size, when clicked on a freshly created project ('ToolsQA_Export_1790772024380').</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>The 'Export' action correctly downloaded 'ToolsQA_Export_1790770675458.xlsx' (2952 bytes).</t>
+          <t>The 'Export' action correctly downloaded 'ToolsQA_Export_1790772024380.xlsx' (2951 bytes).</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">

</xml_diff>